<commit_message>
updated march close, finished assignment
</commit_message>
<xml_diff>
--- a/submissions/excel/excel_07_march_close.xlsx
+++ b/submissions/excel/excel_07_march_close.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\idynamics-training\idynamics-analyst-training\submissions\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E8352FE-A36F-407E-8745-6255AB43FE01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B449E4D3-67EF-45BC-A4E2-8D96B96627E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Historical Baseline" sheetId="1" r:id="rId1"/>
@@ -1332,7 +1332,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1702" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1702" uniqueCount="698">
   <si>
     <t>HISTORICAL BASELINE — 2024 &amp; 2025 ACTUALS</t>
   </si>
@@ -3423,6 +3423,9 @@
   </si>
   <si>
     <t>February finished with a Closing MRR of $150,306. This is $1,764 above what we expected to have currently and has driven EBITDA to $30,214 which is $235 more than our current forecast and provides a margin of 20.1% compared to the planned 20.2%.</t>
+  </si>
+  <si>
+    <t>March 2026 — SaaS KPIs</t>
   </si>
 </sst>
 </file>
@@ -4278,16 +4281,7 @@
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="175" fontId="16" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -4306,6 +4300,15 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -4313,20 +4316,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="28">
-    <dxf>
-      <numFmt numFmtId="22" formatCode="mmm/yy"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFEBF3FB"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -4600,6 +4589,19 @@
       <numFmt numFmtId="22" formatCode="mmm/yy"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="22" formatCode="mmm/yy"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i/>
@@ -4616,6 +4618,16 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFEBF3FB"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -4684,15 +4696,6 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4707,16 +4710,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{33C032D8-7D31-427B-B687-D6ED9274A891}" name="KPI_Tracker" displayName="KPI_Tracker" ref="A3:E16" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{33C032D8-7D31-427B-B687-D6ED9274A891}" name="KPI_Tracker" displayName="KPI_Tracker" ref="A3:E16" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A3:E16" xr:uid="{33C032D8-7D31-427B-B687-D6ED9274A891}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C557A6FD-F6C3-489A-869B-8E7220ED2F0F}" name="Metric" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{C8637273-2623-450B-8EC2-77599710AE46}" name="Jan 2026" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{36B839F2-DBCF-48CC-AD60-ACF3D6D67A87}" name="Feb 2026" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{CF28127B-1023-4FAA-8F51-4A1CC9FF9128}" name="Mar 2026" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{C557A6FD-F6C3-489A-869B-8E7220ED2F0F}" name="Metric" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{C8637273-2623-450B-8EC2-77599710AE46}" name="Jan 2026" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{36B839F2-DBCF-48CC-AD60-ACF3D6D67A87}" name="Feb 2026" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{CF28127B-1023-4FAA-8F51-4A1CC9FF9128}" name="Mar 2026" dataDxfId="22">
       <calculatedColumnFormula>'Mar 2026 A vs F'!B30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7BB998DD-A48B-4270-BB7C-2C1D3FA186B2}" name="Q1 2026" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{7BB998DD-A48B-4270-BB7C-2C1D3FA186B2}" name="Q1 2026" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4726,11 +4729,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0792567E-A03E-4943-98E4-EB876B9B20D6}" name="WaterfallData" displayName="WaterfallData" ref="A1:E22" totalsRowShown="0">
   <autoFilter ref="A1:E22" xr:uid="{0792567E-A03E-4943-98E4-EB876B9B20D6}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E535E1E4-A65E-480E-B37A-792FC0723850}" name="Month" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{E535E1E4-A65E-480E-B37A-792FC0723850}" name="Month" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{AF51F227-B625-4255-94A7-6199B7D7DAD1}" name="Movement"/>
-    <tableColumn id="3" xr3:uid="{72A4FA60-7150-4102-88DE-5B089CAE1D25}" name="Actual" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{69CC0EB6-9154-4E79-8DD0-FAB442AC9657}" name="Forecast" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{4D5B15AB-1D25-4871-B2A0-95F16E574BA9}" name="Variance" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{72A4FA60-7150-4102-88DE-5B089CAE1D25}" name="Actual" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{69CC0EB6-9154-4E79-8DD0-FAB442AC9657}" name="Forecast" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{4D5B15AB-1D25-4871-B2A0-95F16E574BA9}" name="Variance" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4745,8 +4748,8 @@
     <tableColumn id="3" xr3:uid="{3945ECD4-BB6F-4E5B-9B54-0517BF942829}" name="customer_id"/>
     <tableColumn id="4" xr3:uid="{82CA9B0A-4810-468C-8854-3017D97B8592}" name="company_name"/>
     <tableColumn id="5" xr3:uid="{30A8D838-4B8E-4217-8666-E0DF4BB06955}" name="region"/>
-    <tableColumn id="6" xr3:uid="{D841C5AC-D4B5-409A-8CFA-53443E346DCF}" name="month" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{6DBCDEDE-28AB-45B0-93DD-BA33B3BFB675}" name="event_date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{D841C5AC-D4B5-409A-8CFA-53443E346DCF}" name="month" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{6DBCDEDE-28AB-45B0-93DD-BA33B3BFB675}" name="event_date" dataDxfId="15"/>
     <tableColumn id="8" xr3:uid="{C44CB2B9-5967-4692-A03A-7AF3E634A147}" name="event_type"/>
     <tableColumn id="9" xr3:uid="{47B2CD92-F52F-435B-8F19-D30BF4C73CE3}" name="old_value"/>
     <tableColumn id="10" xr3:uid="{5E6457F7-8D2B-4A6E-BB02-89A98B1FF9A9}" name="new_value"/>
@@ -4760,7 +4763,7 @@
     <tableColumn id="18" xr3:uid="{1FFE8D74-8F15-43CF-B8E5-E408F0044790}" name="movement">
       <calculatedColumnFormula array="1">_xlfn.IFS(H2="created", "New", H2="cancelled", "Churned", AND(H2="seats_change", J2 &gt; I2), "Expansion", AND(H2="seats_change", J2 &lt; I2), "Contraction", AND(H2="price_change", J2 &gt; I2), "Expansion", AND(H2="price_change", J2 &lt; I2), "Contraction", H2="plan_upgrade", "Expansion", H2="plan_downgrade", "Contraction", H2="discount_added", "Contraction")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{543176F6-F2BB-4A01-87F5-5C68A679C2B3}" name="mrr_delta" dataDxfId="16">
+    <tableColumn id="19" xr3:uid="{543176F6-F2BB-4A01-87F5-5C68A679C2B3}" name="mrr_delta" dataDxfId="14">
       <calculatedColumnFormula array="1">IF(N2="Monthly",_xlfn.IFS(H2="created",O2*P2*(1-Q2/100),H2="cancelled",-(O2*P2*(1-Q2/100)),H2="seats_change",(J2-I2)*P2*(1-Q2/100),H2="price_change",(J2-I2)*O2*(1-Q2/100),H2="discount_added",-(O2*P2*(J2-I2)/100),H2="plan_upgrade",O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100),H2="plan_downgrade",O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100)),_xlfn.IFS(H2="created",O2*P2*(1-Q2/100)/12,H2="cancelled",-(O2*P2*(1-Q2/100))/12,H2="seats_change",(J2-I2)*P2*(1-Q2/100)/12,H2="price_change",(J2-I2)*O2*(1-Q2/100)/12,H2="plan_upgrade",(O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100))/12,H2="plan_downgrade",(O2*(_xlfn.XLOOKUP(J2,$M:$M,$P:$P)-_xlfn.XLOOKUP(I2,$M:$M,$P:$P))*(1-Q2/100))/12,H2="discount_added",-(O2*P2*(J2-I2)/100)/12))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4769,19 +4772,19 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{539C435F-C1A6-4146-89EF-73537E96D5A1}" name="SMSpend" displayName="SMSpend" ref="A66:J80" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{539C435F-C1A6-4146-89EF-73537E96D5A1}" name="SMSpend" displayName="SMSpend" ref="A66:J80" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A66:J80" xr:uid="{B4D1F123-2972-489C-8FEC-9C6D26BDA440}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{428B9524-495F-4624-8292-AC7281BC37CF}" name="Month" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{A39BE488-44BB-4D32-8BC9-2CAD0287B7FB}" name="Sales Comp" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{5A5033F7-6D0F-4017-B24D-2EF30AF0C04A}" name="Marketing Comp" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{221D6297-6EAF-44F9-9192-FCE924DEAE38}" name="Paid Ads" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{DDDAF5EF-D699-4B54-AE9C-1DE1AE53E1FA}" name="Content &amp; SEO" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{C06DAFB6-3F41-4AB7-AC72-F2CD13738214}" name="Partner Commissions" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{B2373C96-3DA9-4205-B260-ECD2E8248D4F}" name="Tools &amp; Software" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{4C8B3A2D-C15B-426C-8B89-E7B5EA3AC7A8}" name="Events" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{591DAA16-7C9D-4A8A-8098-00ABCE2C68AB}" name="Total S&amp;M" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{27267743-1105-471C-A056-7EE8466EDA53}" name="New Customers" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{428B9524-495F-4624-8292-AC7281BC37CF}" name="Month" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{A39BE488-44BB-4D32-8BC9-2CAD0287B7FB}" name="Sales Comp" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{5A5033F7-6D0F-4017-B24D-2EF30AF0C04A}" name="Marketing Comp" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{221D6297-6EAF-44F9-9192-FCE924DEAE38}" name="Paid Ads" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{DDDAF5EF-D699-4B54-AE9C-1DE1AE53E1FA}" name="Content &amp; SEO" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{C06DAFB6-3F41-4AB7-AC72-F2CD13738214}" name="Partner Commissions" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B2373C96-3DA9-4205-B260-ECD2E8248D4F}" name="Tools &amp; Software" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{4C8B3A2D-C15B-426C-8B89-E7B5EA3AC7A8}" name="Events" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{591DAA16-7C9D-4A8A-8098-00ABCE2C68AB}" name="Total S&amp;M" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{27267743-1105-471C-A056-7EE8466EDA53}" name="New Customers" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4793,8 +4796,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{01F66372-C956-4E27-89CF-1874F2147DCD}" name="plan_name"/>
     <tableColumn id="2" xr3:uid="{CCAD8762-EF12-4CFA-B5B5-C51B5EADA2B4}" name="monthly_price"/>
-    <tableColumn id="3" xr3:uid="{C40B4B1D-B122-4F11-B805-69D33B9BC9E8}" name="monthly_cost" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{9C412AFC-8F05-4E39-B8E1-9E65F1E3A073}" name="gross_margin" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{C40B4B1D-B122-4F11-B805-69D33B9BC9E8}" name="monthly_cost" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9C412AFC-8F05-4E39-B8E1-9E65F1E3A073}" name="gross_margin" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6340,30 +6343,30 @@
       <c r="A47" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="177" t="s">
+      <c r="B47" s="194" t="s">
         <v>311</v>
       </c>
-      <c r="C47" s="177"/>
-      <c r="D47" s="177"/>
-      <c r="E47" s="177"/>
-      <c r="F47" s="177"/>
-      <c r="G47" s="177"/>
-      <c r="H47" s="177"/>
-      <c r="I47" s="177"/>
+      <c r="C47" s="194"/>
+      <c r="D47" s="194"/>
+      <c r="E47" s="194"/>
+      <c r="F47" s="194"/>
+      <c r="G47" s="194"/>
+      <c r="H47" s="194"/>
+      <c r="I47" s="194"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="177" t="s">
+      <c r="B49" s="194" t="s">
         <v>312</v>
       </c>
-      <c r="C49" s="177"/>
-      <c r="D49" s="177"/>
-      <c r="E49" s="177"/>
-      <c r="F49" s="177"/>
-      <c r="G49" s="177"/>
-      <c r="H49" s="177"/>
+      <c r="C49" s="194"/>
+      <c r="D49" s="194"/>
+      <c r="E49" s="194"/>
+      <c r="F49" s="194"/>
+      <c r="G49" s="194"/>
+      <c r="H49" s="194"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6483,7 +6486,7 @@
         <v>8615</v>
       </c>
       <c r="H4" s="38">
-        <f t="shared" ref="H4:H29" si="1">B4+G4</f>
+        <f t="shared" ref="H4:H28" si="1">B4+G4</f>
         <v>14415</v>
       </c>
     </row>
@@ -8623,107 +8626,107 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C19" s="182">
+      <c r="C19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;B15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;B15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;B15)</f>
         <v>2</v>
       </c>
-      <c r="D19" s="182">
+      <c r="D19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;C15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;C15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;C15)</f>
         <v>4</v>
       </c>
-      <c r="E19" s="182">
+      <c r="E19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;D15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;D15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;D15)</f>
         <v>6</v>
       </c>
-      <c r="F19" s="182">
+      <c r="F19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;E15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;E15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;E15)</f>
         <v>9</v>
       </c>
-      <c r="G19" s="182">
+      <c r="G19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;F15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;F15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;F15)</f>
         <v>11</v>
       </c>
-      <c r="H19" s="182">
+      <c r="H19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;G15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;G15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;G15)</f>
         <v>13</v>
       </c>
-      <c r="I19" s="182">
+      <c r="I19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;H15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;H15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;H15)</f>
         <v>15</v>
       </c>
-      <c r="J19" s="182">
+      <c r="J19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;I15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;I15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;I15)</f>
         <v>17</v>
       </c>
-      <c r="K19" s="182">
+      <c r="K19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;J15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;J15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;J15)</f>
         <v>20</v>
       </c>
-      <c r="L19" s="182">
+      <c r="L19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;K15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;K15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;K15)</f>
         <v>22</v>
       </c>
-      <c r="M19" s="182">
+      <c r="M19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;L15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;L15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;L15)</f>
         <v>23</v>
       </c>
-      <c r="N19" s="182">
+      <c r="N19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;M15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;M15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;M15)</f>
         <v>25</v>
       </c>
-      <c r="O19" s="182">
+      <c r="O19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;N15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;N15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;N15)</f>
         <v>26</v>
       </c>
-      <c r="P19" s="182">
+      <c r="P19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;O15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;O15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;O15)</f>
         <v>28</v>
       </c>
-      <c r="Q19" s="182">
+      <c r="Q19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;P15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;P15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;P15)</f>
         <v>31</v>
       </c>
-      <c r="R19" s="182">
+      <c r="R19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Q15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Q15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Q15)</f>
         <v>33</v>
       </c>
-      <c r="S19" s="182">
+      <c r="S19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;R15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;R15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;R15)</f>
         <v>36</v>
       </c>
-      <c r="T19" s="182">
+      <c r="T19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;S15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;S15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;S15)</f>
         <v>37</v>
       </c>
-      <c r="U19" s="182">
+      <c r="U19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;T15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;T15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;T15)</f>
         <v>37</v>
       </c>
-      <c r="V19" s="182">
+      <c r="V19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;U15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;U15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;U15)</f>
         <v>37</v>
       </c>
-      <c r="W19" s="182">
+      <c r="W19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;V15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;V15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;V15)</f>
         <v>37</v>
       </c>
-      <c r="X19" s="182">
+      <c r="X19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;W15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;W15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;W15)</f>
         <v>38</v>
       </c>
-      <c r="Y19" s="182">
+      <c r="Y19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;X15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;X15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;X15)</f>
         <v>38</v>
       </c>
-      <c r="Z19" s="182">
+      <c r="Z19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Y15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Y15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Y15)</f>
         <v>38</v>
       </c>
-      <c r="AA19" s="182">
+      <c r="AA19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Z15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Z15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;Z15)</f>
         <v>39</v>
       </c>
-      <c r="AB19" s="182">
+      <c r="AB19" s="177">
         <f>COUNTIFS(Engine!$T$2:$T$102,1,Engine!$F$2:$F$102,"&lt;="&amp;AA15)+COUNTIFS(Engine!$V$2:$V$102,1,Engine!$F$2:$F$102,"&lt;="&amp;AA15)-COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,"&lt;="&amp;AA15)</f>
         <v>41</v>
       </c>
@@ -8732,111 +8735,111 @@
       <c r="A20" s="45" t="s">
         <v>178</v>
       </c>
-      <c r="B20" s="182">
+      <c r="B20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,B15)</f>
         <v>0</v>
       </c>
-      <c r="C20" s="182">
+      <c r="C20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,C15)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="182">
+      <c r="D20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,D15)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="182">
+      <c r="E20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,E15)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="182">
+      <c r="F20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,F15)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="182">
+      <c r="G20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,G15)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="182">
+      <c r="H20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,H15)</f>
         <v>0</v>
       </c>
-      <c r="I20" s="182">
+      <c r="I20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,I15)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="182">
+      <c r="J20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,J15)</f>
         <v>0</v>
       </c>
-      <c r="K20" s="182">
+      <c r="K20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,K15)</f>
         <v>0</v>
       </c>
-      <c r="L20" s="182">
+      <c r="L20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,L15)</f>
         <v>1</v>
       </c>
-      <c r="M20" s="182">
+      <c r="M20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,M15)</f>
         <v>0</v>
       </c>
-      <c r="N20" s="182">
+      <c r="N20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,N15)</f>
         <v>1</v>
       </c>
-      <c r="O20" s="182">
+      <c r="O20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,O15)</f>
         <v>0</v>
       </c>
-      <c r="P20" s="182">
+      <c r="P20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,P15)</f>
         <v>0</v>
       </c>
-      <c r="Q20" s="182">
+      <c r="Q20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,Q15)</f>
         <v>0</v>
       </c>
-      <c r="R20" s="182">
+      <c r="R20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,R15)</f>
         <v>0</v>
       </c>
-      <c r="S20" s="182">
+      <c r="S20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,S15)</f>
         <v>1</v>
       </c>
-      <c r="T20" s="182">
+      <c r="T20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,T15)</f>
         <v>0</v>
       </c>
-      <c r="U20" s="182">
+      <c r="U20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,U15)</f>
         <v>0</v>
       </c>
-      <c r="V20" s="182">
+      <c r="V20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,V15)</f>
         <v>0</v>
       </c>
-      <c r="W20" s="182">
+      <c r="W20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,W15)</f>
         <v>0</v>
       </c>
-      <c r="X20" s="182">
+      <c r="X20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,X15)</f>
         <v>0</v>
       </c>
-      <c r="Y20" s="182">
+      <c r="Y20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,Y15)</f>
         <v>0</v>
       </c>
-      <c r="Z20" s="182">
+      <c r="Z20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,Z15)</f>
         <v>0</v>
       </c>
-      <c r="AA20" s="182">
+      <c r="AA20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,AA15)</f>
         <v>0</v>
       </c>
-      <c r="AB20" s="182">
+      <c r="AB20" s="177">
         <f>COUNTIFS(Engine!$U$2:$U$102,1,Engine!$F$2:$F$102,AB15)</f>
         <v>0</v>
       </c>
@@ -9319,7 +9322,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="28">
-        <f t="shared" ref="E27:AB27" si="6">AVERAGE(D21:F21)</f>
+        <f t="shared" ref="F27:AB27" si="6">AVERAGE(D21:F21)</f>
         <v>0</v>
       </c>
       <c r="G27" s="28">
@@ -9786,35 +9789,35 @@
       </c>
     </row>
     <row r="34" spans="1:27" ht="80" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="179" t="s">
+      <c r="A34" s="196" t="s">
         <v>188</v>
       </c>
-      <c r="B34" s="180"/>
-      <c r="C34" s="180"/>
-      <c r="D34" s="180"/>
-      <c r="E34" s="180"/>
-      <c r="F34" s="180"/>
-      <c r="G34" s="180"/>
-      <c r="H34" s="180"/>
-      <c r="I34" s="180"/>
-      <c r="J34" s="180"/>
-      <c r="K34" s="180"/>
-      <c r="L34" s="180"/>
-      <c r="M34" s="180"/>
-      <c r="N34" s="180"/>
-      <c r="O34" s="180"/>
-      <c r="P34" s="180"/>
-      <c r="Q34" s="180"/>
-      <c r="R34" s="180"/>
-      <c r="S34" s="180"/>
-      <c r="T34" s="180"/>
-      <c r="U34" s="180"/>
-      <c r="V34" s="180"/>
-      <c r="W34" s="180"/>
-      <c r="X34" s="180"/>
-      <c r="Y34" s="180"/>
-      <c r="Z34" s="180"/>
-      <c r="AA34" s="180"/>
+      <c r="B34" s="197"/>
+      <c r="C34" s="197"/>
+      <c r="D34" s="197"/>
+      <c r="E34" s="197"/>
+      <c r="F34" s="197"/>
+      <c r="G34" s="197"/>
+      <c r="H34" s="197"/>
+      <c r="I34" s="197"/>
+      <c r="J34" s="197"/>
+      <c r="K34" s="197"/>
+      <c r="L34" s="197"/>
+      <c r="M34" s="197"/>
+      <c r="N34" s="197"/>
+      <c r="O34" s="197"/>
+      <c r="P34" s="197"/>
+      <c r="Q34" s="197"/>
+      <c r="R34" s="197"/>
+      <c r="S34" s="197"/>
+      <c r="T34" s="197"/>
+      <c r="U34" s="197"/>
+      <c r="V34" s="197"/>
+      <c r="W34" s="197"/>
+      <c r="X34" s="197"/>
+      <c r="Y34" s="197"/>
+      <c r="Z34" s="197"/>
+      <c r="AA34" s="197"/>
     </row>
     <row r="35" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:27" x14ac:dyDescent="0.35">
@@ -9823,35 +9826,35 @@
       </c>
     </row>
     <row r="37" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="179" t="s">
+      <c r="A37" s="196" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="180"/>
-      <c r="C37" s="180"/>
-      <c r="D37" s="180"/>
-      <c r="E37" s="180"/>
-      <c r="F37" s="180"/>
-      <c r="G37" s="180"/>
-      <c r="H37" s="180"/>
-      <c r="I37" s="180"/>
-      <c r="J37" s="180"/>
-      <c r="K37" s="180"/>
-      <c r="L37" s="180"/>
-      <c r="M37" s="180"/>
-      <c r="N37" s="180"/>
-      <c r="O37" s="180"/>
-      <c r="P37" s="180"/>
-      <c r="Q37" s="180"/>
-      <c r="R37" s="180"/>
-      <c r="S37" s="180"/>
-      <c r="T37" s="180"/>
-      <c r="U37" s="180"/>
-      <c r="V37" s="180"/>
-      <c r="W37" s="180"/>
-      <c r="X37" s="180"/>
-      <c r="Y37" s="180"/>
-      <c r="Z37" s="180"/>
-      <c r="AA37" s="180"/>
+      <c r="B37" s="197"/>
+      <c r="C37" s="197"/>
+      <c r="D37" s="197"/>
+      <c r="E37" s="197"/>
+      <c r="F37" s="197"/>
+      <c r="G37" s="197"/>
+      <c r="H37" s="197"/>
+      <c r="I37" s="197"/>
+      <c r="J37" s="197"/>
+      <c r="K37" s="197"/>
+      <c r="L37" s="197"/>
+      <c r="M37" s="197"/>
+      <c r="N37" s="197"/>
+      <c r="O37" s="197"/>
+      <c r="P37" s="197"/>
+      <c r="Q37" s="197"/>
+      <c r="R37" s="197"/>
+      <c r="S37" s="197"/>
+      <c r="T37" s="197"/>
+      <c r="U37" s="197"/>
+      <c r="V37" s="197"/>
+      <c r="W37" s="197"/>
+      <c r="X37" s="197"/>
+      <c r="Y37" s="197"/>
+      <c r="Z37" s="197"/>
+      <c r="AA37" s="197"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10575,18 +10578,18 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="181" t="s">
+      <c r="A64" s="198" t="s">
         <v>256</v>
       </c>
-      <c r="B64" s="181"/>
-      <c r="C64" s="181"/>
-      <c r="D64" s="181"/>
-      <c r="E64" s="181"/>
-      <c r="F64" s="181"/>
-      <c r="G64" s="181"/>
-      <c r="H64" s="181"/>
-      <c r="I64" s="181"/>
-      <c r="J64" s="181"/>
+      <c r="B64" s="198"/>
+      <c r="C64" s="198"/>
+      <c r="D64" s="198"/>
+      <c r="E64" s="198"/>
+      <c r="F64" s="198"/>
+      <c r="G64" s="198"/>
+      <c r="H64" s="198"/>
+      <c r="I64" s="198"/>
+      <c r="J64" s="198"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
@@ -13488,20 +13491,19 @@
         <v>144779.5</v>
       </c>
       <c r="C3" s="129">
-        <f>'Jan 2026 A vs F '!B9</f>
-        <v>144779.5</v>
+        <v>146831.04999999999</v>
       </c>
       <c r="D3" s="129">
         <f t="shared" ref="D3:D10" si="0">B3-C3</f>
-        <v>0</v>
+        <v>-2051.5499999999884</v>
       </c>
       <c r="E3" s="130">
         <f>IFERROR(B3/C3-1, 0)</f>
-        <v>0</v>
+        <v>-1.397218095218955E-2</v>
       </c>
       <c r="F3" s="131" t="str" cm="1">
         <f t="array" ref="F3">_xlfn.IFS(D3&lt;0, "U", D3&gt;0, "F", D3=0, "-")</f>
-        <v>-</v>
+        <v>U</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -13594,8 +13596,8 @@
         <v>-0.37722575391680269</v>
       </c>
       <c r="F7" s="134" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.IFS(D7&gt;0, "U", D7&lt;0, "F", D7=0, "-")</f>
-        <v>U</v>
+        <f t="array" ref="F7">_xlfn.IFS(D7&gt;0, "F", D7&lt;0, "U", D7=0, "-")</f>
+        <v>F</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -13633,19 +13635,19 @@
       </c>
       <c r="C9" s="140">
         <f>C3+C8</f>
-        <v>148541.05083333334</v>
+        <v>150592.60083333333</v>
       </c>
       <c r="D9" s="140">
         <f t="shared" si="0"/>
-        <v>1764.4491666666581</v>
+        <v>-287.10083333333023</v>
       </c>
       <c r="E9" s="141">
         <f>B9/C9-1</f>
-        <v>1.1878528910142183E-2</v>
+        <v>-1.9064737028552381E-3</v>
       </c>
       <c r="F9" s="142" t="str" cm="1">
         <f t="array" ref="F9">_xlfn.IFS(D9&lt;0, "U", D9&gt;0, "F", D9=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -13658,19 +13660,19 @@
       </c>
       <c r="C10" s="143">
         <f>C9*12</f>
-        <v>1782492.61</v>
+        <v>1807111.21</v>
       </c>
       <c r="D10" s="143">
         <f t="shared" si="0"/>
-        <v>21173.389999999898</v>
+        <v>-3445.2099999999627</v>
       </c>
       <c r="E10" s="144">
         <f>B10/C10-1</f>
-        <v>1.1878528910142183E-2</v>
+        <v>-1.9064737028552381E-3</v>
       </c>
       <c r="F10" s="145" t="str" cm="1">
         <f t="array" ref="F10">_xlfn.IFS(D10&lt;0, "U", D10&gt;0, "F", D10=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -13716,19 +13718,19 @@
       </c>
       <c r="C14" s="132">
         <f>C9</f>
-        <v>148541.05083333334</v>
+        <v>150592.60083333333</v>
       </c>
       <c r="D14" s="132">
         <f t="shared" ref="D14:D23" si="1">B14-C14</f>
-        <v>1764.4491666666581</v>
+        <v>-287.10083333333023</v>
       </c>
       <c r="E14" s="133">
         <f t="shared" ref="E14:E23" si="2">B14/C14-1</f>
-        <v>1.1878528910142183E-2</v>
+        <v>-1.9064737028552381E-3</v>
       </c>
       <c r="F14" s="131" t="str" cm="1">
         <f t="array" ref="F14">_xlfn.IFS(D14&lt;0, "U", D14&gt;0, "F", D14=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>120</v>
@@ -13744,19 +13746,19 @@
       </c>
       <c r="C15" s="132">
         <f>C14*0.3</f>
-        <v>44562.31525</v>
+        <v>45177.780249999996</v>
       </c>
       <c r="D15" s="132">
         <f t="shared" si="1"/>
-        <v>529.33475000000908</v>
+        <v>-86.130249999987427</v>
       </c>
       <c r="E15" s="133">
         <f t="shared" si="2"/>
-        <v>1.1878528910142405E-2</v>
+        <v>-1.9064737028550161E-3</v>
       </c>
       <c r="F15" s="131" t="str" cm="1">
         <f t="array" ref="F15">_xlfn.IFS(D15&gt;0, "U", D15&lt;0, "F", D15=0, "-")</f>
-        <v>U</v>
+        <v>F</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>121</v>
@@ -13772,19 +13774,19 @@
       </c>
       <c r="C16" s="147">
         <f>C14-C15</f>
-        <v>103978.73558333334</v>
+        <v>105414.82058333333</v>
       </c>
       <c r="D16" s="147">
         <f t="shared" si="1"/>
-        <v>1235.114416666649</v>
+        <v>-200.9705833333428</v>
       </c>
       <c r="E16" s="148">
         <f t="shared" si="2"/>
-        <v>1.1878528910142183E-2</v>
+        <v>-1.9064737028553491E-3</v>
       </c>
       <c r="F16" s="149" t="str" cm="1">
         <f t="array" ref="F16">_xlfn.IFS(D16&lt;0, "U", D16&gt;0, "F", D16=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>122</v>
@@ -13938,19 +13940,19 @@
       </c>
       <c r="C22" s="153">
         <f>C16-C21</f>
-        <v>29978.735583333342</v>
+        <v>31414.820583333334</v>
       </c>
       <c r="D22" s="153">
         <f t="shared" si="1"/>
-        <v>235.11441666664905</v>
+        <v>-1200.9705833333428</v>
       </c>
       <c r="E22" s="154">
         <f t="shared" si="2"/>
-        <v>7.842706241331987E-3</v>
+        <v>-3.8229426781144826E-2</v>
       </c>
       <c r="F22" s="155" t="str" cm="1">
         <f t="array" ref="F22">_xlfn.IFS(D22&lt;0, "U", D22&gt;0, "F", D22=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>125</v>
@@ -13966,15 +13968,15 @@
       </c>
       <c r="C23" s="133">
         <f>C22/C14</f>
-        <v>0.20182121652667054</v>
+        <v>0.20860799540942476</v>
       </c>
       <c r="D23" s="133">
         <f t="shared" si="1"/>
-        <v>-8.0495298342034283E-4</v>
+        <v>-7.591731866174567E-3</v>
       </c>
       <c r="E23" s="133">
         <f t="shared" si="2"/>
-        <v>-3.9884458000676304E-3</v>
+        <v>-3.6392334106248647E-2</v>
       </c>
       <c r="F23" s="131" t="str" cm="1">
         <f t="array" ref="F23">IFERROR(_xlfn.IFS(D23&lt;0, "U", D23&gt;0, "F", D23=0, "-"), "-")</f>
@@ -14397,20 +14399,19 @@
         <v>150305.5</v>
       </c>
       <c r="C3" s="129">
-        <f>'Jan 2026 A vs F '!B9</f>
-        <v>144779.5</v>
+        <v>150592.6</v>
       </c>
       <c r="D3" s="129">
         <f t="shared" ref="D3:D10" si="0">B3-C3</f>
-        <v>5526</v>
+        <v>-287.10000000000582</v>
       </c>
       <c r="E3" s="130">
         <f>IFERROR(B3/C3-1, 0)</f>
-        <v>3.8168387099002166E-2</v>
+        <v>-1.9064681797114069E-3</v>
       </c>
       <c r="F3" s="131" t="str" cm="1">
         <f t="array" ref="F3">_xlfn.IFS(D3&lt;0, "U", D3&gt;0, "F", D3=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -14503,8 +14504,8 @@
         <v>-1</v>
       </c>
       <c r="F7" s="134" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.IFS(D7&gt;0, "U", D7&lt;0, "F", D7=0, "-")</f>
-        <v>U</v>
+        <f t="array" ref="F7">_xlfn.IFS(D7&gt;0, "F", D7&lt;0, "U", D7=0, "-")</f>
+        <v>F</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -14542,19 +14543,19 @@
       </c>
       <c r="C9" s="140">
         <f>C3+C8</f>
-        <v>148541.05083333334</v>
+        <v>154354.15083333335</v>
       </c>
       <c r="D9" s="140">
         <f t="shared" si="0"/>
-        <v>4944.4491666666581</v>
+        <v>-868.65083333334769</v>
       </c>
       <c r="E9" s="141">
         <f>B9/C9-1</f>
-        <v>3.3286752308050227E-2</v>
+        <v>-5.6276480330696987E-3</v>
       </c>
       <c r="F9" s="142" t="str" cm="1">
         <f t="array" ref="F9">_xlfn.IFS(D9&lt;0, "U", D9&gt;0, "F", D9=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -14567,19 +14568,19 @@
       </c>
       <c r="C10" s="143">
         <f>C9*12</f>
-        <v>1782492.61</v>
+        <v>1852249.81</v>
       </c>
       <c r="D10" s="143">
         <f t="shared" si="0"/>
-        <v>59333.389999999898</v>
+        <v>-10423.810000000056</v>
       </c>
       <c r="E10" s="144">
         <f>B10/C10-1</f>
-        <v>3.3286752308050227E-2</v>
+        <v>-5.6276480330695877E-3</v>
       </c>
       <c r="F10" s="145" t="str" cm="1">
         <f t="array" ref="F10">_xlfn.IFS(D10&lt;0, "U", D10&gt;0, "F", D10=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
@@ -14625,19 +14626,19 @@
       </c>
       <c r="C14" s="132">
         <f>C9</f>
-        <v>148541.05083333334</v>
+        <v>154354.15083333335</v>
       </c>
       <c r="D14" s="132">
         <f t="shared" ref="D14:D23" si="1">B14-C14</f>
-        <v>4944.4491666666581</v>
+        <v>-868.65083333334769</v>
       </c>
       <c r="E14" s="133">
         <f t="shared" ref="E14:E23" si="2">B14/C14-1</f>
-        <v>3.3286752308050227E-2</v>
+        <v>-5.6276480330696987E-3</v>
       </c>
       <c r="F14" s="131" t="str" cm="1">
         <f t="array" ref="F14">_xlfn.IFS(D14&lt;0, "U", D14&gt;0, "F", D14=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>120</v>
@@ -14653,19 +14654,19 @@
       </c>
       <c r="C15" s="132">
         <f>C14*0.3</f>
-        <v>44562.31525</v>
+        <v>46306.24525</v>
       </c>
       <c r="D15" s="132">
         <f t="shared" si="1"/>
-        <v>1483.3347500000091</v>
+        <v>-260.59524999999121</v>
       </c>
       <c r="E15" s="133">
         <f t="shared" si="2"/>
-        <v>3.3286752308050449E-2</v>
+        <v>-5.6276480330693657E-3</v>
       </c>
       <c r="F15" s="131" t="str" cm="1">
         <f t="array" ref="F15">_xlfn.IFS(D15&gt;0, "U", D15&lt;0, "F", D15=0, "-")</f>
-        <v>U</v>
+        <v>F</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>121</v>
@@ -14681,19 +14682,19 @@
       </c>
       <c r="C16" s="147">
         <f>C14-C15</f>
-        <v>103978.73558333334</v>
+        <v>108047.90558333334</v>
       </c>
       <c r="D16" s="147">
         <f t="shared" si="1"/>
-        <v>3461.114416666649</v>
+        <v>-608.0555833333492</v>
       </c>
       <c r="E16" s="148">
         <f t="shared" si="2"/>
-        <v>3.3286752308050005E-2</v>
+        <v>-5.6276480330696987E-3</v>
       </c>
       <c r="F16" s="149" t="str" cm="1">
         <f t="array" ref="F16">_xlfn.IFS(D16&lt;0, "U", D16&gt;0, "F", D16=0, "-")</f>
-        <v>F</v>
+        <v>U</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>122</v>
@@ -14708,7 +14709,7 @@
       </c>
       <c r="C17" s="156">
         <f>C16/C14</f>
-        <v>0.70000000000000007</v>
+        <v>0.7</v>
       </c>
       <c r="D17" s="156">
         <f t="shared" si="1"/>
@@ -14845,15 +14846,15 @@
       </c>
       <c r="C22" s="153">
         <f>C16-C21</f>
-        <v>29978.735583333342</v>
+        <v>34047.90558333334</v>
       </c>
       <c r="D22" s="153">
         <f t="shared" si="1"/>
-        <v>4461.114416666649</v>
+        <v>391.9444166666508</v>
       </c>
       <c r="E22" s="154">
         <f t="shared" si="2"/>
-        <v>0.14880929198184067</v>
+        <v>1.1511557317596344E-2</v>
       </c>
       <c r="F22" s="155" t="str" cm="1">
         <f t="array" ref="F22">_xlfn.IFS(D22&lt;0, "U", D22&gt;0, "F", D22=0, "-")</f>
@@ -14873,15 +14874,15 @@
       </c>
       <c r="C23" s="133">
         <f>C22/C14</f>
-        <v>0.20182121652667054</v>
+        <v>0.22058302546134426</v>
       </c>
       <c r="D23" s="133">
         <f t="shared" si="1"/>
-        <v>2.2563823102480035E-2</v>
+        <v>3.8020141678063168E-3</v>
       </c>
       <c r="E23" s="133">
         <f t="shared" si="2"/>
-        <v>0.11180104594948892</v>
+        <v>1.7236204643827469E-2</v>
       </c>
       <c r="F23" s="131" t="str" cm="1">
         <f t="array" ref="F23">IFERROR(_xlfn.IFS(D23&lt;0, "U", D23&gt;0, "F", D23=0, "-"), "-")</f>
@@ -14893,7 +14894,7 @@
     </row>
     <row r="27" spans="1:8" ht="17" x14ac:dyDescent="0.4">
       <c r="A27" s="160" t="s">
-        <v>658</v>
+        <v>697</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
@@ -15071,8 +15072,8 @@
         <v>660</v>
       </c>
       <c r="B40" s="164">
-        <f>IFERROR(IF(('Jan 2026 A vs F '!B46/'Jan 2026 A vs F '!B47+B39)=0,"—",('Jan 2026 A vs F '!B46+B37)/('Jan 2026 A vs F '!B46/'Jan 2026 A vs F '!B47+B39)),"—")</f>
-        <v>19666.666666666668</v>
+        <f>IFERROR(IF(('Jan 2026 A vs F '!B46/'Jan 2026 A vs F '!B47+'Feb 2026 A vs F'!B39+B39)=0,"—",('Jan 2026 A vs F '!B46+'Feb 2026 A vs F'!B37+B37)/('Jan 2026 A vs F '!B46/'Jan 2026 A vs F '!B47+'Feb 2026 A vs F'!B39+B39)),"—")</f>
+        <v>18000</v>
       </c>
       <c r="C40" s="124" t="s">
         <v>629</v>
@@ -15500,11 +15501,11 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="178" t="s">
+      <c r="A18" s="195" t="s">
         <v>645</v>
       </c>
-      <c r="B18" s="178"/>
-      <c r="C18" s="178"/>
+      <c r="B18" s="195"/>
+      <c r="C18" s="195"/>
       <c r="D18" s="123"/>
       <c r="E18" s="123"/>
     </row>
@@ -15551,7 +15552,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="198">
+      <c r="A2" s="193">
         <v>46023</v>
       </c>
       <c r="B2" t="s">
@@ -15571,7 +15572,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="198">
+      <c r="A3" s="193">
         <v>46023</v>
       </c>
       <c r="B3" t="s">
@@ -15591,7 +15592,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="198">
+      <c r="A4" s="193">
         <v>46023</v>
       </c>
       <c r="B4" t="s">
@@ -15611,7 +15612,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="198">
+      <c r="A5" s="193">
         <v>46023</v>
       </c>
       <c r="B5" t="s">
@@ -15631,7 +15632,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="198">
+      <c r="A6" s="193">
         <v>46023</v>
       </c>
       <c r="B6" t="s">
@@ -15651,7 +15652,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="198">
+      <c r="A7" s="193">
         <v>46023</v>
       </c>
       <c r="B7" t="s">
@@ -15671,7 +15672,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="198">
+      <c r="A8" s="193">
         <v>46023</v>
       </c>
       <c r="B8" t="s">
@@ -15691,7 +15692,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="198" t="str">
+      <c r="A9" s="193" t="str">
         <f t="shared" ref="A9:A15" si="0">TEXT(DATE(2026,2,1),"mmm-yy")</f>
         <v>Feb-26</v>
       </c>
@@ -15704,15 +15705,15 @@
       </c>
       <c r="D9" s="175">
         <f>'Feb 2026 A vs F'!C3</f>
-        <v>144779.5</v>
+        <v>146831.04999999999</v>
       </c>
       <c r="E9" s="175">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>-2051.5499999999884</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="198" t="str">
+      <c r="A10" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15733,7 +15734,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="198" t="str">
+      <c r="A11" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15754,7 +15755,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="198" t="str">
+      <c r="A12" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15775,7 +15776,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="198" t="str">
+      <c r="A13" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15796,7 +15797,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="198" t="str">
+      <c r="A14" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15817,7 +15818,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="198" t="str">
+      <c r="A15" s="193" t="str">
         <f t="shared" si="0"/>
         <v>Feb-26</v>
       </c>
@@ -15830,72 +15831,72 @@
       </c>
       <c r="D15" s="169">
         <f>'Feb 2026 A vs F'!C9</f>
-        <v>148541.05083333334</v>
+        <v>150592.60083333333</v>
       </c>
       <c r="E15" s="169">
         <f>C15-D15</f>
-        <v>1764.4491666666581</v>
+        <v>-287.10083333333023</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A16" s="193" t="str">
+        <f t="shared" ref="A16:A22" si="1">TEXT(DATE(2026,3,1),"mmm-yy")</f>
         <v>Mar-26</v>
       </c>
-      <c r="B16" s="195" t="s">
+      <c r="B16" s="190" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="196">
+      <c r="C16" s="191">
         <f>'Mar 2026 A vs F'!B3</f>
         <v>150305.5</v>
       </c>
-      <c r="D16" s="196">
+      <c r="D16" s="191">
         <f>'Mar 2026 A vs F'!C3</f>
-        <v>144779.5</v>
-      </c>
-      <c r="E16" s="197">
+        <v>150592.6</v>
+      </c>
+      <c r="E16" s="192">
         <f>'Mar 2026 A vs F'!D3</f>
-        <v>5526</v>
+        <v>-287.10000000000582</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A17" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B17" s="192" t="s">
+      <c r="B17" s="187" t="s">
         <v>650</v>
       </c>
-      <c r="C17" s="193">
+      <c r="C17" s="188">
         <f>'Mar 2026 A vs F'!B4</f>
         <v>3000</v>
       </c>
-      <c r="D17" s="193">
+      <c r="D17" s="188">
         <f>'Mar 2026 A vs F'!C4</f>
         <v>4000</v>
       </c>
-      <c r="E17" s="194">
+      <c r="E17" s="189">
         <f>'Mar 2026 A vs F'!D4</f>
         <v>-1000</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A18" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B18" s="183" t="s">
+      <c r="B18" s="178" t="s">
         <v>651</v>
       </c>
-      <c r="C18" s="190">
+      <c r="C18" s="185">
         <f>'Mar 2026 A vs F'!B5</f>
         <v>180</v>
       </c>
-      <c r="D18" s="190">
+      <c r="D18" s="185">
         <f>'Mar 2026 A vs F'!C5</f>
         <v>715.34749999999997</v>
       </c>
-      <c r="E18" s="185">
+      <c r="E18" s="180">
         <f>'Mar 2026 A vs F'!D5</f>
         <v>-535.34749999999997</v>
       </c>
@@ -15904,87 +15905,87 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A19" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B19" s="188" t="s">
+      <c r="B19" s="183" t="s">
         <v>652</v>
       </c>
-      <c r="C19" s="191">
+      <c r="C19" s="186">
         <f>'Mar 2026 A vs F'!B6</f>
         <v>0</v>
       </c>
-      <c r="D19" s="191">
+      <c r="D19" s="186">
         <f>'Mar 2026 A vs F'!C6</f>
         <v>0</v>
       </c>
-      <c r="E19" s="189">
+      <c r="E19" s="184">
         <f>D19-C19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A20" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B20" s="183" t="s">
+      <c r="B20" s="178" t="s">
         <v>653</v>
       </c>
-      <c r="C20" s="190">
+      <c r="C20" s="185">
         <f>'Mar 2026 A vs F'!B7</f>
         <v>0</v>
       </c>
-      <c r="D20" s="190">
+      <c r="D20" s="185">
         <f>'Mar 2026 A vs F'!C7</f>
         <v>953.79666666666662</v>
       </c>
-      <c r="E20" s="185">
+      <c r="E20" s="180">
         <f>'Mar 2026 A vs F'!D7</f>
         <v>953.79666666666662</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A21" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B21" s="188" t="s">
+      <c r="B21" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="191">
+      <c r="C21" s="186">
         <f>'Mar 2026 A vs F'!B8</f>
         <v>3180</v>
       </c>
-      <c r="D21" s="191">
+      <c r="D21" s="186">
         <f>'Mar 2026 A vs F'!C8</f>
         <v>3761.5508333333332</v>
       </c>
-      <c r="E21" s="189">
+      <c r="E21" s="184">
         <f>'Mar 2026 A vs F'!D8</f>
         <v>-581.55083333333323</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="198" t="str">
-        <f>TEXT(DATE(2026,3,1),"mmm-yy")</f>
+      <c r="A22" s="193" t="str">
+        <f t="shared" si="1"/>
         <v>Mar-26</v>
       </c>
-      <c r="B22" s="184" t="s">
+      <c r="B22" s="179" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="187">
+      <c r="C22" s="182">
         <f>'Mar 2026 A vs F'!B9</f>
         <v>153485.5</v>
       </c>
-      <c r="D22" s="187">
+      <c r="D22" s="182">
         <f>'Mar 2026 A vs F'!C9</f>
-        <v>148541.05083333334</v>
-      </c>
-      <c r="E22" s="186">
+        <v>154354.15083333335</v>
+      </c>
+      <c r="E22" s="181">
         <f>'Mar 2026 A vs F'!D9</f>
-        <v>4944.4491666666581</v>
+        <v>-868.65083333334769</v>
       </c>
     </row>
   </sheetData>
@@ -16145,11 +16146,11 @@
         <v>1</v>
       </c>
       <c r="U2">
-        <f>IF(H2&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F2)-COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F2)=0,1,0))</f>
+        <f t="shared" ref="U2:U33" si="0">IF(H2&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F2)-COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F2)=0,1,0))</f>
         <v>0</v>
       </c>
       <c r="V2">
-        <f>IF(AND(H2="created",T2=0,COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F2)&gt;0,COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F2)-COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F2)=0),1,0)</f>
+        <f t="shared" ref="V2:V33" si="1">IF(AND(H2="created",T2=0,COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F2)&gt;0,COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F2)-COUNTIFS($C$2:$C$102,$C2,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F2)=0),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -16206,11 +16207,11 @@
         <v>1</v>
       </c>
       <c r="U3">
-        <f>IF(H3&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C3,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F3)-COUNTIFS($C$2:$C$102,$C3,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F3)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V3">
-        <f>IF(AND(H3="created",T3=0,COUNTIFS($C$2:$C$102,$C3,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F3)&gt;0,COUNTIFS($C$2:$C$102,$C3,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F3)-COUNTIFS($C$2:$C$102,$C3,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F3)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16267,11 +16268,11 @@
         <v>1</v>
       </c>
       <c r="U4">
-        <f>IF(H4&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C4,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F4)-COUNTIFS($C$2:$C$102,$C4,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F4)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V4">
-        <f>IF(AND(H4="created",T4=0,COUNTIFS($C$2:$C$102,$C4,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F4)&gt;0,COUNTIFS($C$2:$C$102,$C4,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F4)-COUNTIFS($C$2:$C$102,$C4,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F4)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16328,11 +16329,11 @@
         <v>1</v>
       </c>
       <c r="U5">
-        <f>IF(H5&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C5,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F5)-COUNTIFS($C$2:$C$102,$C5,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F5)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V5">
-        <f>IF(AND(H5="created",T5=0,COUNTIFS($C$2:$C$102,$C5,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F5)&gt;0,COUNTIFS($C$2:$C$102,$C5,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F5)-COUNTIFS($C$2:$C$102,$C5,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F5)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16389,11 +16390,11 @@
         <v>0</v>
       </c>
       <c r="U6">
-        <f>IF(H6&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C6,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F6)-COUNTIFS($C$2:$C$102,$C6,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F6)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V6">
-        <f>IF(AND(H6="created",T6=0,COUNTIFS($C$2:$C$102,$C6,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F6)&gt;0,COUNTIFS($C$2:$C$102,$C6,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F6)-COUNTIFS($C$2:$C$102,$C6,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F6)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16450,11 +16451,11 @@
         <v>1</v>
       </c>
       <c r="U7">
-        <f>IF(H7&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C7,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F7)-COUNTIFS($C$2:$C$102,$C7,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F7)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V7">
-        <f>IF(AND(H7="created",T7=0,COUNTIFS($C$2:$C$102,$C7,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F7)&gt;0,COUNTIFS($C$2:$C$102,$C7,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F7)-COUNTIFS($C$2:$C$102,$C7,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F7)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16511,11 +16512,11 @@
         <v>1</v>
       </c>
       <c r="U8">
-        <f>IF(H8&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C8,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F8)-COUNTIFS($C$2:$C$102,$C8,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F8)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V8">
-        <f>IF(AND(H8="created",T8=0,COUNTIFS($C$2:$C$102,$C8,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F8)&gt;0,COUNTIFS($C$2:$C$102,$C8,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F8)-COUNTIFS($C$2:$C$102,$C8,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F8)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16572,11 +16573,11 @@
         <v>1</v>
       </c>
       <c r="U9">
-        <f>IF(H9&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C9,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F9)-COUNTIFS($C$2:$C$102,$C9,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F9)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V9">
-        <f>IF(AND(H9="created",T9=0,COUNTIFS($C$2:$C$102,$C9,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F9)&gt;0,COUNTIFS($C$2:$C$102,$C9,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F9)-COUNTIFS($C$2:$C$102,$C9,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F9)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16633,11 +16634,11 @@
         <v>0</v>
       </c>
       <c r="U10">
-        <f>IF(H10&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C10,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F10)-COUNTIFS($C$2:$C$102,$C10,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F10)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V10">
-        <f>IF(AND(H10="created",T10=0,COUNTIFS($C$2:$C$102,$C10,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F10)&gt;0,COUNTIFS($C$2:$C$102,$C10,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F10)-COUNTIFS($C$2:$C$102,$C10,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F10)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16694,11 +16695,11 @@
         <v>1</v>
       </c>
       <c r="U11">
-        <f>IF(H11&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C11,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F11)-COUNTIFS($C$2:$C$102,$C11,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F11)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V11">
-        <f>IF(AND(H11="created",T11=0,COUNTIFS($C$2:$C$102,$C11,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F11)&gt;0,COUNTIFS($C$2:$C$102,$C11,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F11)-COUNTIFS($C$2:$C$102,$C11,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F11)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16755,11 +16756,11 @@
         <v>1</v>
       </c>
       <c r="U12">
-        <f>IF(H12&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C12,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F12)-COUNTIFS($C$2:$C$102,$C12,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F12)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V12">
-        <f>IF(AND(H12="created",T12=0,COUNTIFS($C$2:$C$102,$C12,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F12)&gt;0,COUNTIFS($C$2:$C$102,$C12,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F12)-COUNTIFS($C$2:$C$102,$C12,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F12)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16816,11 +16817,11 @@
         <v>1</v>
       </c>
       <c r="U13">
-        <f>IF(H13&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C13,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F13)-COUNTIFS($C$2:$C$102,$C13,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F13)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V13">
-        <f>IF(AND(H13="created",T13=0,COUNTIFS($C$2:$C$102,$C13,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F13)&gt;0,COUNTIFS($C$2:$C$102,$C13,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F13)-COUNTIFS($C$2:$C$102,$C13,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F13)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16877,11 +16878,11 @@
         <v>1</v>
       </c>
       <c r="U14">
-        <f>IF(H14&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C14,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F14)-COUNTIFS($C$2:$C$102,$C14,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F14)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V14">
-        <f>IF(AND(H14="created",T14=0,COUNTIFS($C$2:$C$102,$C14,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F14)&gt;0,COUNTIFS($C$2:$C$102,$C14,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F14)-COUNTIFS($C$2:$C$102,$C14,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F14)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16938,11 +16939,11 @@
         <v>1</v>
       </c>
       <c r="U15">
-        <f>IF(H15&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C15,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F15)-COUNTIFS($C$2:$C$102,$C15,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F15)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V15">
-        <f>IF(AND(H15="created",T15=0,COUNTIFS($C$2:$C$102,$C15,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F15)&gt;0,COUNTIFS($C$2:$C$102,$C15,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F15)-COUNTIFS($C$2:$C$102,$C15,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F15)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -16999,11 +17000,11 @@
         <v>0</v>
       </c>
       <c r="U16">
-        <f>IF(H16&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C16,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F16)-COUNTIFS($C$2:$C$102,$C16,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F16)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V16">
-        <f>IF(AND(H16="created",T16=0,COUNTIFS($C$2:$C$102,$C16,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F16)&gt;0,COUNTIFS($C$2:$C$102,$C16,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F16)-COUNTIFS($C$2:$C$102,$C16,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F16)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17060,11 +17061,11 @@
         <v>1</v>
       </c>
       <c r="U17">
-        <f>IF(H17&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C17,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F17)-COUNTIFS($C$2:$C$102,$C17,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F17)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V17">
-        <f>IF(AND(H17="created",T17=0,COUNTIFS($C$2:$C$102,$C17,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F17)&gt;0,COUNTIFS($C$2:$C$102,$C17,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F17)-COUNTIFS($C$2:$C$102,$C17,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F17)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17121,11 +17122,11 @@
         <v>1</v>
       </c>
       <c r="U18">
-        <f>IF(H18&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C18,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F18)-COUNTIFS($C$2:$C$102,$C18,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F18)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V18">
-        <f>IF(AND(H18="created",T18=0,COUNTIFS($C$2:$C$102,$C18,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F18)&gt;0,COUNTIFS($C$2:$C$102,$C18,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F18)-COUNTIFS($C$2:$C$102,$C18,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F18)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17182,11 +17183,11 @@
         <v>0</v>
       </c>
       <c r="U19">
-        <f>IF(H19&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C19,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F19)-COUNTIFS($C$2:$C$102,$C19,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F19)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V19">
-        <f>IF(AND(H19="created",T19=0,COUNTIFS($C$2:$C$102,$C19,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F19)&gt;0,COUNTIFS($C$2:$C$102,$C19,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F19)-COUNTIFS($C$2:$C$102,$C19,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F19)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17243,11 +17244,11 @@
         <v>1</v>
       </c>
       <c r="U20">
-        <f>IF(H20&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C20,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F20)-COUNTIFS($C$2:$C$102,$C20,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F20)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V20">
-        <f>IF(AND(H20="created",T20=0,COUNTIFS($C$2:$C$102,$C20,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F20)&gt;0,COUNTIFS($C$2:$C$102,$C20,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F20)-COUNTIFS($C$2:$C$102,$C20,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F20)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17304,11 +17305,11 @@
         <v>0</v>
       </c>
       <c r="U21">
-        <f>IF(H21&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C21,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F21)-COUNTIFS($C$2:$C$102,$C21,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F21)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V21">
-        <f>IF(AND(H21="created",T21=0,COUNTIFS($C$2:$C$102,$C21,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F21)&gt;0,COUNTIFS($C$2:$C$102,$C21,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F21)-COUNTIFS($C$2:$C$102,$C21,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F21)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17365,11 +17366,11 @@
         <v>1</v>
       </c>
       <c r="U22">
-        <f>IF(H22&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C22,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F22)-COUNTIFS($C$2:$C$102,$C22,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F22)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V22">
-        <f>IF(AND(H22="created",T22=0,COUNTIFS($C$2:$C$102,$C22,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F22)&gt;0,COUNTIFS($C$2:$C$102,$C22,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F22)-COUNTIFS($C$2:$C$102,$C22,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F22)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17426,11 +17427,11 @@
         <v>1</v>
       </c>
       <c r="U23">
-        <f>IF(H23&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C23,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F23)-COUNTIFS($C$2:$C$102,$C23,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F23)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V23">
-        <f>IF(AND(H23="created",T23=0,COUNTIFS($C$2:$C$102,$C23,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F23)&gt;0,COUNTIFS($C$2:$C$102,$C23,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F23)-COUNTIFS($C$2:$C$102,$C23,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F23)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17499,11 +17500,11 @@
         <v>0</v>
       </c>
       <c r="U24">
-        <f>IF(H24&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C24,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F24)-COUNTIFS($C$2:$C$102,$C24,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F24)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V24">
-        <f>IF(AND(H24="created",T24=0,COUNTIFS($C$2:$C$102,$C24,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F24)&gt;0,COUNTIFS($C$2:$C$102,$C24,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F24)-COUNTIFS($C$2:$C$102,$C24,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F24)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17560,11 +17561,11 @@
         <v>1</v>
       </c>
       <c r="U25">
-        <f>IF(H25&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C25,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F25)-COUNTIFS($C$2:$C$102,$C25,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F25)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V25">
-        <f>IF(AND(H25="created",T25=0,COUNTIFS($C$2:$C$102,$C25,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F25)&gt;0,COUNTIFS($C$2:$C$102,$C25,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F25)-COUNTIFS($C$2:$C$102,$C25,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F25)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17621,11 +17622,11 @@
         <v>0</v>
       </c>
       <c r="U26">
-        <f>IF(H26&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C26,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F26)-COUNTIFS($C$2:$C$102,$C26,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F26)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V26">
-        <f>IF(AND(H26="created",T26=0,COUNTIFS($C$2:$C$102,$C26,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F26)&gt;0,COUNTIFS($C$2:$C$102,$C26,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F26)-COUNTIFS($C$2:$C$102,$C26,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F26)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17682,11 +17683,11 @@
         <v>1</v>
       </c>
       <c r="U27">
-        <f>IF(H27&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C27,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F27)-COUNTIFS($C$2:$C$102,$C27,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F27)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V27">
-        <f>IF(AND(H27="created",T27=0,COUNTIFS($C$2:$C$102,$C27,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F27)&gt;0,COUNTIFS($C$2:$C$102,$C27,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F27)-COUNTIFS($C$2:$C$102,$C27,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F27)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17743,11 +17744,11 @@
         <v>0</v>
       </c>
       <c r="U28">
-        <f>IF(H28&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C28,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F28)-COUNTIFS($C$2:$C$102,$C28,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F28)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V28">
-        <f>IF(AND(H28="created",T28=0,COUNTIFS($C$2:$C$102,$C28,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F28)&gt;0,COUNTIFS($C$2:$C$102,$C28,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F28)-COUNTIFS($C$2:$C$102,$C28,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F28)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17804,11 +17805,11 @@
         <v>1</v>
       </c>
       <c r="U29">
-        <f>IF(H29&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C29,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F29)-COUNTIFS($C$2:$C$102,$C29,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F29)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V29">
-        <f>IF(AND(H29="created",T29=0,COUNTIFS($C$2:$C$102,$C29,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F29)&gt;0,COUNTIFS($C$2:$C$102,$C29,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F29)-COUNTIFS($C$2:$C$102,$C29,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F29)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17865,11 +17866,11 @@
         <v>0</v>
       </c>
       <c r="U30">
-        <f>IF(H30&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C30,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F30)-COUNTIFS($C$2:$C$102,$C30,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F30)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V30">
-        <f>IF(AND(H30="created",T30=0,COUNTIFS($C$2:$C$102,$C30,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F30)&gt;0,COUNTIFS($C$2:$C$102,$C30,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F30)-COUNTIFS($C$2:$C$102,$C30,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F30)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17926,11 +17927,11 @@
         <v>1</v>
       </c>
       <c r="U31">
-        <f>IF(H31&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C31,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F31)-COUNTIFS($C$2:$C$102,$C31,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F31)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V31">
-        <f>IF(AND(H31="created",T31=0,COUNTIFS($C$2:$C$102,$C31,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F31)&gt;0,COUNTIFS($C$2:$C$102,$C31,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F31)-COUNTIFS($C$2:$C$102,$C31,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F31)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -17987,11 +17988,11 @@
         <v>1</v>
       </c>
       <c r="U32">
-        <f>IF(H32&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C32,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F32)-COUNTIFS($C$2:$C$102,$C32,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F32)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V32">
-        <f>IF(AND(H32="created",T32=0,COUNTIFS($C$2:$C$102,$C32,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F32)&gt;0,COUNTIFS($C$2:$C$102,$C32,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F32)-COUNTIFS($C$2:$C$102,$C32,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F32)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -18048,11 +18049,11 @@
         <v>0</v>
       </c>
       <c r="U33">
-        <f>IF(H33&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C33,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F33)-COUNTIFS($C$2:$C$102,$C33,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F33)=0,1,0))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V33">
-        <f>IF(AND(H33="created",T33=0,COUNTIFS($C$2:$C$102,$C33,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F33)&gt;0,COUNTIFS($C$2:$C$102,$C33,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F33)-COUNTIFS($C$2:$C$102,$C33,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F33)=0),1,0)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -18109,11 +18110,11 @@
         <v>1</v>
       </c>
       <c r="U34">
-        <f>IF(H34&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F34)-COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F34)=0,1,0))</f>
+        <f t="shared" ref="U34:U65" si="2">IF(H34&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F34)-COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F34)=0,1,0))</f>
         <v>0</v>
       </c>
       <c r="V34">
-        <f>IF(AND(H34="created",T34=0,COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F34)&gt;0,COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F34)-COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F34)=0),1,0)</f>
+        <f t="shared" ref="V34:V65" si="3">IF(AND(H34="created",T34=0,COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F34)&gt;0,COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F34)-COUNTIFS($C$2:$C$102,$C34,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F34)=0),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -18182,11 +18183,11 @@
         <v>0</v>
       </c>
       <c r="U35">
-        <f>IF(H35&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C35,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F35)-COUNTIFS($C$2:$C$102,$C35,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F35)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="V35">
-        <f>IF(AND(H35="created",T35=0,COUNTIFS($C$2:$C$102,$C35,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F35)&gt;0,COUNTIFS($C$2:$C$102,$C35,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F35)-COUNTIFS($C$2:$C$102,$C35,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F35)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18243,11 +18244,11 @@
         <v>1</v>
       </c>
       <c r="U36">
-        <f>IF(H36&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C36,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F36)-COUNTIFS($C$2:$C$102,$C36,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F36)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V36">
-        <f>IF(AND(H36="created",T36=0,COUNTIFS($C$2:$C$102,$C36,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F36)&gt;0,COUNTIFS($C$2:$C$102,$C36,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F36)-COUNTIFS($C$2:$C$102,$C36,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F36)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18304,11 +18305,11 @@
         <v>1</v>
       </c>
       <c r="U37">
-        <f>IF(H37&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C37,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F37)-COUNTIFS($C$2:$C$102,$C37,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F37)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V37">
-        <f>IF(AND(H37="created",T37=0,COUNTIFS($C$2:$C$102,$C37,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F37)&gt;0,COUNTIFS($C$2:$C$102,$C37,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F37)-COUNTIFS($C$2:$C$102,$C37,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F37)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18365,11 +18366,11 @@
         <v>0</v>
       </c>
       <c r="U38">
-        <f>IF(H38&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C38,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F38)-COUNTIFS($C$2:$C$102,$C38,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F38)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V38">
-        <f>IF(AND(H38="created",T38=0,COUNTIFS($C$2:$C$102,$C38,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F38)&gt;0,COUNTIFS($C$2:$C$102,$C38,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F38)-COUNTIFS($C$2:$C$102,$C38,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F38)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18426,11 +18427,11 @@
         <v>0</v>
       </c>
       <c r="U39">
-        <f>IF(H39&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C39,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F39)-COUNTIFS($C$2:$C$102,$C39,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F39)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V39">
-        <f>IF(AND(H39="created",T39=0,COUNTIFS($C$2:$C$102,$C39,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F39)&gt;0,COUNTIFS($C$2:$C$102,$C39,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F39)-COUNTIFS($C$2:$C$102,$C39,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F39)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18499,11 +18500,11 @@
         <v>0</v>
       </c>
       <c r="U40">
-        <f>IF(H40&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C40,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F40)-COUNTIFS($C$2:$C$102,$C40,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F40)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V40">
-        <f>IF(AND(H40="created",T40=0,COUNTIFS($C$2:$C$102,$C40,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F40)&gt;0,COUNTIFS($C$2:$C$102,$C40,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F40)-COUNTIFS($C$2:$C$102,$C40,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F40)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18560,11 +18561,11 @@
         <v>1</v>
       </c>
       <c r="U41">
-        <f>IF(H41&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C41,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F41)-COUNTIFS($C$2:$C$102,$C41,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F41)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V41">
-        <f>IF(AND(H41="created",T41=0,COUNTIFS($C$2:$C$102,$C41,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F41)&gt;0,COUNTIFS($C$2:$C$102,$C41,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F41)-COUNTIFS($C$2:$C$102,$C41,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F41)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18621,11 +18622,11 @@
         <v>1</v>
       </c>
       <c r="U42">
-        <f>IF(H42&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C42,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F42)-COUNTIFS($C$2:$C$102,$C42,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F42)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V42">
-        <f>IF(AND(H42="created",T42=0,COUNTIFS($C$2:$C$102,$C42,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F42)&gt;0,COUNTIFS($C$2:$C$102,$C42,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F42)-COUNTIFS($C$2:$C$102,$C42,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F42)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18694,11 +18695,11 @@
         <v>0</v>
       </c>
       <c r="U43">
-        <f>IF(H43&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C43,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F43)-COUNTIFS($C$2:$C$102,$C43,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F43)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V43">
-        <f>IF(AND(H43="created",T43=0,COUNTIFS($C$2:$C$102,$C43,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F43)&gt;0,COUNTIFS($C$2:$C$102,$C43,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F43)-COUNTIFS($C$2:$C$102,$C43,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F43)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18767,11 +18768,11 @@
         <v>0</v>
       </c>
       <c r="U44">
-        <f>IF(H44&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C44,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F44)-COUNTIFS($C$2:$C$102,$C44,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F44)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="V44">
-        <f>IF(AND(H44="created",T44=0,COUNTIFS($C$2:$C$102,$C44,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F44)&gt;0,COUNTIFS($C$2:$C$102,$C44,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F44)-COUNTIFS($C$2:$C$102,$C44,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F44)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18828,11 +18829,11 @@
         <v>1</v>
       </c>
       <c r="U45">
-        <f>IF(H45&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C45,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F45)-COUNTIFS($C$2:$C$102,$C45,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F45)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V45">
-        <f>IF(AND(H45="created",T45=0,COUNTIFS($C$2:$C$102,$C45,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F45)&gt;0,COUNTIFS($C$2:$C$102,$C45,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F45)-COUNTIFS($C$2:$C$102,$C45,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F45)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18889,11 +18890,11 @@
         <v>0</v>
       </c>
       <c r="U46">
-        <f>IF(H46&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C46,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F46)-COUNTIFS($C$2:$C$102,$C46,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F46)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V46">
-        <f>IF(AND(H46="created",T46=0,COUNTIFS($C$2:$C$102,$C46,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F46)&gt;0,COUNTIFS($C$2:$C$102,$C46,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F46)-COUNTIFS($C$2:$C$102,$C46,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F46)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -18950,11 +18951,11 @@
         <v>0</v>
       </c>
       <c r="U47">
-        <f>IF(H47&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C47,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F47)-COUNTIFS($C$2:$C$102,$C47,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F47)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V47">
-        <f>IF(AND(H47="created",T47=0,COUNTIFS($C$2:$C$102,$C47,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F47)&gt;0,COUNTIFS($C$2:$C$102,$C47,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F47)-COUNTIFS($C$2:$C$102,$C47,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F47)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19011,11 +19012,11 @@
         <v>1</v>
       </c>
       <c r="U48">
-        <f>IF(H48&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C48,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F48)-COUNTIFS($C$2:$C$102,$C48,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F48)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V48">
-        <f>IF(AND(H48="created",T48=0,COUNTIFS($C$2:$C$102,$C48,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F48)&gt;0,COUNTIFS($C$2:$C$102,$C48,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F48)-COUNTIFS($C$2:$C$102,$C48,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F48)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19072,11 +19073,11 @@
         <v>0</v>
       </c>
       <c r="U49">
-        <f>IF(H49&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C49,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F49)-COUNTIFS($C$2:$C$102,$C49,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F49)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V49">
-        <f>IF(AND(H49="created",T49=0,COUNTIFS($C$2:$C$102,$C49,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F49)&gt;0,COUNTIFS($C$2:$C$102,$C49,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F49)-COUNTIFS($C$2:$C$102,$C49,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F49)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19133,11 +19134,11 @@
         <v>0</v>
       </c>
       <c r="U50">
-        <f>IF(H50&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C50,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F50)-COUNTIFS($C$2:$C$102,$C50,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F50)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V50">
-        <f>IF(AND(H50="created",T50=0,COUNTIFS($C$2:$C$102,$C50,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F50)&gt;0,COUNTIFS($C$2:$C$102,$C50,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F50)-COUNTIFS($C$2:$C$102,$C50,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F50)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19194,11 +19195,11 @@
         <v>1</v>
       </c>
       <c r="U51">
-        <f>IF(H51&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C51,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F51)-COUNTIFS($C$2:$C$102,$C51,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F51)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V51">
-        <f>IF(AND(H51="created",T51=0,COUNTIFS($C$2:$C$102,$C51,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F51)&gt;0,COUNTIFS($C$2:$C$102,$C51,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F51)-COUNTIFS($C$2:$C$102,$C51,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F51)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19255,11 +19256,11 @@
         <v>1</v>
       </c>
       <c r="U52">
-        <f>IF(H52&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C52,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F52)-COUNTIFS($C$2:$C$102,$C52,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F52)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V52">
-        <f>IF(AND(H52="created",T52=0,COUNTIFS($C$2:$C$102,$C52,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F52)&gt;0,COUNTIFS($C$2:$C$102,$C52,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F52)-COUNTIFS($C$2:$C$102,$C52,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F52)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19316,11 +19317,11 @@
         <v>0</v>
       </c>
       <c r="U53">
-        <f>IF(H53&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C53,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F53)-COUNTIFS($C$2:$C$102,$C53,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F53)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V53">
-        <f>IF(AND(H53="created",T53=0,COUNTIFS($C$2:$C$102,$C53,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F53)&gt;0,COUNTIFS($C$2:$C$102,$C53,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F53)-COUNTIFS($C$2:$C$102,$C53,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F53)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19389,11 +19390,11 @@
         <v>0</v>
       </c>
       <c r="U54">
-        <f>IF(H54&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C54,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F54)-COUNTIFS($C$2:$C$102,$C54,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F54)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V54">
-        <f>IF(AND(H54="created",T54=0,COUNTIFS($C$2:$C$102,$C54,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F54)&gt;0,COUNTIFS($C$2:$C$102,$C54,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F54)-COUNTIFS($C$2:$C$102,$C54,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F54)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19450,11 +19451,11 @@
         <v>0</v>
       </c>
       <c r="U55">
-        <f>IF(H55&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C55,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F55)-COUNTIFS($C$2:$C$102,$C55,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F55)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V55">
-        <f>IF(AND(H55="created",T55=0,COUNTIFS($C$2:$C$102,$C55,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F55)&gt;0,COUNTIFS($C$2:$C$102,$C55,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F55)-COUNTIFS($C$2:$C$102,$C55,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F55)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19523,11 +19524,11 @@
         <v>0</v>
       </c>
       <c r="U56">
-        <f>IF(H56&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C56,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F56)-COUNTIFS($C$2:$C$102,$C56,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F56)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V56">
-        <f>IF(AND(H56="created",T56=0,COUNTIFS($C$2:$C$102,$C56,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F56)&gt;0,COUNTIFS($C$2:$C$102,$C56,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F56)-COUNTIFS($C$2:$C$102,$C56,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F56)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19584,11 +19585,11 @@
         <v>1</v>
       </c>
       <c r="U57">
-        <f>IF(H57&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C57,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F57)-COUNTIFS($C$2:$C$102,$C57,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F57)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V57">
-        <f>IF(AND(H57="created",T57=0,COUNTIFS($C$2:$C$102,$C57,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F57)&gt;0,COUNTIFS($C$2:$C$102,$C57,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F57)-COUNTIFS($C$2:$C$102,$C57,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F57)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19657,11 +19658,11 @@
         <v>0</v>
       </c>
       <c r="U58">
-        <f>IF(H58&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C58,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F58)-COUNTIFS($C$2:$C$102,$C58,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F58)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V58">
-        <f>IF(AND(H58="created",T58=0,COUNTIFS($C$2:$C$102,$C58,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F58)&gt;0,COUNTIFS($C$2:$C$102,$C58,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F58)-COUNTIFS($C$2:$C$102,$C58,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F58)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19718,11 +19719,11 @@
         <v>1</v>
       </c>
       <c r="U59">
-        <f>IF(H59&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C59,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F59)-COUNTIFS($C$2:$C$102,$C59,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F59)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V59">
-        <f>IF(AND(H59="created",T59=0,COUNTIFS($C$2:$C$102,$C59,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F59)&gt;0,COUNTIFS($C$2:$C$102,$C59,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F59)-COUNTIFS($C$2:$C$102,$C59,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F59)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19791,11 +19792,11 @@
         <v>0</v>
       </c>
       <c r="U60">
-        <f>IF(H60&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C60,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F60)-COUNTIFS($C$2:$C$102,$C60,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F60)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V60">
-        <f>IF(AND(H60="created",T60=0,COUNTIFS($C$2:$C$102,$C60,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F60)&gt;0,COUNTIFS($C$2:$C$102,$C60,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F60)-COUNTIFS($C$2:$C$102,$C60,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F60)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19852,11 +19853,11 @@
         <v>1</v>
       </c>
       <c r="U61">
-        <f>IF(H61&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C61,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F61)-COUNTIFS($C$2:$C$102,$C61,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F61)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V61">
-        <f>IF(AND(H61="created",T61=0,COUNTIFS($C$2:$C$102,$C61,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F61)&gt;0,COUNTIFS($C$2:$C$102,$C61,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F61)-COUNTIFS($C$2:$C$102,$C61,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F61)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19925,11 +19926,11 @@
         <v>0</v>
       </c>
       <c r="U62">
-        <f>IF(H62&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C62,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F62)-COUNTIFS($C$2:$C$102,$C62,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F62)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V62">
-        <f>IF(AND(H62="created",T62=0,COUNTIFS($C$2:$C$102,$C62,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F62)&gt;0,COUNTIFS($C$2:$C$102,$C62,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F62)-COUNTIFS($C$2:$C$102,$C62,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F62)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -19986,11 +19987,11 @@
         <v>0</v>
       </c>
       <c r="U63">
-        <f>IF(H63&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C63,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F63)-COUNTIFS($C$2:$C$102,$C63,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F63)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V63">
-        <f>IF(AND(H63="created",T63=0,COUNTIFS($C$2:$C$102,$C63,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F63)&gt;0,COUNTIFS($C$2:$C$102,$C63,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F63)-COUNTIFS($C$2:$C$102,$C63,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F63)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -20047,11 +20048,11 @@
         <v>1</v>
       </c>
       <c r="U64">
-        <f>IF(H64&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C64,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F64)-COUNTIFS($C$2:$C$102,$C64,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F64)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V64">
-        <f>IF(AND(H64="created",T64=0,COUNTIFS($C$2:$C$102,$C64,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F64)&gt;0,COUNTIFS($C$2:$C$102,$C64,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F64)-COUNTIFS($C$2:$C$102,$C64,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F64)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -20120,11 +20121,11 @@
         <v>0</v>
       </c>
       <c r="U65">
-        <f>IF(H65&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C65,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F65)-COUNTIFS($C$2:$C$102,$C65,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F65)=0,1,0))</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="V65">
-        <f>IF(AND(H65="created",T65=0,COUNTIFS($C$2:$C$102,$C65,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F65)&gt;0,COUNTIFS($C$2:$C$102,$C65,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F65)-COUNTIFS($C$2:$C$102,$C65,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F65)=0),1,0)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -20181,11 +20182,11 @@
         <v>1</v>
       </c>
       <c r="U66">
-        <f>IF(H66&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F66)-COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F66)=0,1,0))</f>
+        <f t="shared" ref="U66:U98" si="4">IF(H66&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F66)-COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F66)=0,1,0))</f>
         <v>0</v>
       </c>
       <c r="V66">
-        <f>IF(AND(H66="created",T66=0,COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F66)&gt;0,COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F66)-COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F66)=0),1,0)</f>
+        <f t="shared" ref="V66:V98" si="5">IF(AND(H66="created",T66=0,COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F66)&gt;0,COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F66)-COUNTIFS($C$2:$C$102,$C66,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F66)=0),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -20245,11 +20246,11 @@
         <v>0</v>
       </c>
       <c r="U67">
-        <f>IF(H67&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C67,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F67)-COUNTIFS($C$2:$C$102,$C67,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F67)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V67">
-        <f>IF(AND(H67="created",T67=0,COUNTIFS($C$2:$C$102,$C67,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F67)&gt;0,COUNTIFS($C$2:$C$102,$C67,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F67)-COUNTIFS($C$2:$C$102,$C67,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F67)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
     </row>
@@ -20306,11 +20307,11 @@
         <v>0</v>
       </c>
       <c r="U68">
-        <f>IF(H68&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C68,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F68)-COUNTIFS($C$2:$C$102,$C68,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F68)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V68">
-        <f>IF(AND(H68="created",T68=0,COUNTIFS($C$2:$C$102,$C68,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F68)&gt;0,COUNTIFS($C$2:$C$102,$C68,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F68)-COUNTIFS($C$2:$C$102,$C68,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F68)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20379,11 +20380,11 @@
         <v>0</v>
       </c>
       <c r="U69">
-        <f>IF(H69&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C69,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F69)-COUNTIFS($C$2:$C$102,$C69,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F69)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V69">
-        <f>IF(AND(H69="created",T69=0,COUNTIFS($C$2:$C$102,$C69,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F69)&gt;0,COUNTIFS($C$2:$C$102,$C69,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F69)-COUNTIFS($C$2:$C$102,$C69,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F69)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20440,11 +20441,11 @@
         <v>1</v>
       </c>
       <c r="U70">
-        <f>IF(H70&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C70,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F70)-COUNTIFS($C$2:$C$102,$C70,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F70)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V70">
-        <f>IF(AND(H70="created",T70=0,COUNTIFS($C$2:$C$102,$C70,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F70)&gt;0,COUNTIFS($C$2:$C$102,$C70,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F70)-COUNTIFS($C$2:$C$102,$C70,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F70)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20513,11 +20514,11 @@
         <v>0</v>
       </c>
       <c r="U71">
-        <f>IF(H71&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C71,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F71)-COUNTIFS($C$2:$C$102,$C71,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F71)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V71">
-        <f>IF(AND(H71="created",T71=0,COUNTIFS($C$2:$C$102,$C71,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F71)&gt;0,COUNTIFS($C$2:$C$102,$C71,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F71)-COUNTIFS($C$2:$C$102,$C71,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F71)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20574,11 +20575,11 @@
         <v>0</v>
       </c>
       <c r="U72">
-        <f>IF(H72&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C72,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F72)-COUNTIFS($C$2:$C$102,$C72,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F72)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V72">
-        <f>IF(AND(H72="created",T72=0,COUNTIFS($C$2:$C$102,$C72,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F72)&gt;0,COUNTIFS($C$2:$C$102,$C72,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F72)-COUNTIFS($C$2:$C$102,$C72,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F72)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20635,11 +20636,11 @@
         <v>1</v>
       </c>
       <c r="U73">
-        <f>IF(H73&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C73,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F73)-COUNTIFS($C$2:$C$102,$C73,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F73)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V73">
-        <f>IF(AND(H73="created",T73=0,COUNTIFS($C$2:$C$102,$C73,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F73)&gt;0,COUNTIFS($C$2:$C$102,$C73,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F73)-COUNTIFS($C$2:$C$102,$C73,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F73)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20708,11 +20709,11 @@
         <v>0</v>
       </c>
       <c r="U74">
-        <f>IF(H74&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C74,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F74)-COUNTIFS($C$2:$C$102,$C74,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F74)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V74">
-        <f>IF(AND(H74="created",T74=0,COUNTIFS($C$2:$C$102,$C74,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F74)&gt;0,COUNTIFS($C$2:$C$102,$C74,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F74)-COUNTIFS($C$2:$C$102,$C74,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F74)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20781,11 +20782,11 @@
         <v>0</v>
       </c>
       <c r="U75">
-        <f>IF(H75&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C75,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F75)-COUNTIFS($C$2:$C$102,$C75,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F75)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V75">
-        <f>IF(AND(H75="created",T75=0,COUNTIFS($C$2:$C$102,$C75,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F75)&gt;0,COUNTIFS($C$2:$C$102,$C75,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F75)-COUNTIFS($C$2:$C$102,$C75,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F75)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20842,11 +20843,11 @@
         <v>1</v>
       </c>
       <c r="U76">
-        <f>IF(H76&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C76,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F76)-COUNTIFS($C$2:$C$102,$C76,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F76)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V76">
-        <f>IF(AND(H76="created",T76=0,COUNTIFS($C$2:$C$102,$C76,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F76)&gt;0,COUNTIFS($C$2:$C$102,$C76,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F76)-COUNTIFS($C$2:$C$102,$C76,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F76)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20915,11 +20916,11 @@
         <v>0</v>
       </c>
       <c r="U77">
-        <f>IF(H77&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C77,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F77)-COUNTIFS($C$2:$C$102,$C77,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F77)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="V77">
-        <f>IF(AND(H77="created",T77=0,COUNTIFS($C$2:$C$102,$C77,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F77)&gt;0,COUNTIFS($C$2:$C$102,$C77,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F77)-COUNTIFS($C$2:$C$102,$C77,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F77)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -20988,11 +20989,11 @@
         <v>0</v>
       </c>
       <c r="U78">
-        <f>IF(H78&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C78,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F78)-COUNTIFS($C$2:$C$102,$C78,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F78)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V78">
-        <f>IF(AND(H78="created",T78=0,COUNTIFS($C$2:$C$102,$C78,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F78)&gt;0,COUNTIFS($C$2:$C$102,$C78,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F78)-COUNTIFS($C$2:$C$102,$C78,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F78)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21061,11 +21062,11 @@
         <v>0</v>
       </c>
       <c r="U79">
-        <f>IF(H79&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C79,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F79)-COUNTIFS($C$2:$C$102,$C79,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F79)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V79">
-        <f>IF(AND(H79="created",T79=0,COUNTIFS($C$2:$C$102,$C79,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F79)&gt;0,COUNTIFS($C$2:$C$102,$C79,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F79)-COUNTIFS($C$2:$C$102,$C79,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F79)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21134,11 +21135,11 @@
         <v>0</v>
       </c>
       <c r="U80">
-        <f>IF(H80&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C80,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F80)-COUNTIFS($C$2:$C$102,$C80,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F80)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V80">
-        <f>IF(AND(H80="created",T80=0,COUNTIFS($C$2:$C$102,$C80,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F80)&gt;0,COUNTIFS($C$2:$C$102,$C80,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F80)-COUNTIFS($C$2:$C$102,$C80,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F80)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21207,11 +21208,11 @@
         <v>0</v>
       </c>
       <c r="U81">
-        <f>IF(H81&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C81,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F81)-COUNTIFS($C$2:$C$102,$C81,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F81)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V81">
-        <f>IF(AND(H81="created",T81=0,COUNTIFS($C$2:$C$102,$C81,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F81)&gt;0,COUNTIFS($C$2:$C$102,$C81,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F81)-COUNTIFS($C$2:$C$102,$C81,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F81)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21280,11 +21281,11 @@
         <v>0</v>
       </c>
       <c r="U82">
-        <f>IF(H82&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C82,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F82)-COUNTIFS($C$2:$C$102,$C82,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F82)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V82">
-        <f>IF(AND(H82="created",T82=0,COUNTIFS($C$2:$C$102,$C82,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F82)&gt;0,COUNTIFS($C$2:$C$102,$C82,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F82)-COUNTIFS($C$2:$C$102,$C82,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F82)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21353,11 +21354,11 @@
         <v>0</v>
       </c>
       <c r="U83">
-        <f>IF(H83&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C83,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F83)-COUNTIFS($C$2:$C$102,$C83,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F83)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V83">
-        <f>IF(AND(H83="created",T83=0,COUNTIFS($C$2:$C$102,$C83,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F83)&gt;0,COUNTIFS($C$2:$C$102,$C83,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F83)-COUNTIFS($C$2:$C$102,$C83,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F83)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21426,11 +21427,11 @@
         <v>0</v>
       </c>
       <c r="U84">
-        <f>IF(H84&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C84,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F84)-COUNTIFS($C$2:$C$102,$C84,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F84)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V84">
-        <f>IF(AND(H84="created",T84=0,COUNTIFS($C$2:$C$102,$C84,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F84)&gt;0,COUNTIFS($C$2:$C$102,$C84,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F84)-COUNTIFS($C$2:$C$102,$C84,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F84)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21499,11 +21500,11 @@
         <v>0</v>
       </c>
       <c r="U85">
-        <f>IF(H85&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C85,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F85)-COUNTIFS($C$2:$C$102,$C85,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F85)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V85">
-        <f>IF(AND(H85="created",T85=0,COUNTIFS($C$2:$C$102,$C85,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F85)&gt;0,COUNTIFS($C$2:$C$102,$C85,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F85)-COUNTIFS($C$2:$C$102,$C85,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F85)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21572,11 +21573,11 @@
         <v>0</v>
       </c>
       <c r="U86">
-        <f>IF(H86&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C86,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F86)-COUNTIFS($C$2:$C$102,$C86,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F86)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V86">
-        <f>IF(AND(H86="created",T86=0,COUNTIFS($C$2:$C$102,$C86,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F86)&gt;0,COUNTIFS($C$2:$C$102,$C86,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F86)-COUNTIFS($C$2:$C$102,$C86,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F86)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21645,11 +21646,11 @@
         <v>0</v>
       </c>
       <c r="U87">
-        <f>IF(H87&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C87,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F87)-COUNTIFS($C$2:$C$102,$C87,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F87)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V87">
-        <f>IF(AND(H87="created",T87=0,COUNTIFS($C$2:$C$102,$C87,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F87)&gt;0,COUNTIFS($C$2:$C$102,$C87,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F87)-COUNTIFS($C$2:$C$102,$C87,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F87)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21718,11 +21719,11 @@
         <v>0</v>
       </c>
       <c r="U88">
-        <f>IF(H88&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C88,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F88)-COUNTIFS($C$2:$C$102,$C88,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F88)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V88">
-        <f>IF(AND(H88="created",T88=0,COUNTIFS($C$2:$C$102,$C88,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F88)&gt;0,COUNTIFS($C$2:$C$102,$C88,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F88)-COUNTIFS($C$2:$C$102,$C88,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F88)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21791,11 +21792,11 @@
         <v>0</v>
       </c>
       <c r="U89">
-        <f>IF(H89&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C89,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F89)-COUNTIFS($C$2:$C$102,$C89,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F89)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V89">
-        <f>IF(AND(H89="created",T89=0,COUNTIFS($C$2:$C$102,$C89,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F89)&gt;0,COUNTIFS($C$2:$C$102,$C89,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F89)-COUNTIFS($C$2:$C$102,$C89,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F89)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -21855,11 +21856,11 @@
         <v>0</v>
       </c>
       <c r="U90">
-        <f>IF(H90&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C90,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F90)-COUNTIFS($C$2:$C$102,$C90,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F90)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V90">
-        <f>IF(AND(H90="created",T90=0,COUNTIFS($C$2:$C$102,$C90,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F90)&gt;0,COUNTIFS($C$2:$C$102,$C90,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F90)-COUNTIFS($C$2:$C$102,$C90,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F90)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
     </row>
@@ -21928,11 +21929,11 @@
         <v>0</v>
       </c>
       <c r="U91">
-        <f>IF(H91&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C91,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F91)-COUNTIFS($C$2:$C$102,$C91,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F91)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V91">
-        <f>IF(AND(H91="created",T91=0,COUNTIFS($C$2:$C$102,$C91,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F91)&gt;0,COUNTIFS($C$2:$C$102,$C91,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F91)-COUNTIFS($C$2:$C$102,$C91,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F91)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22001,11 +22002,11 @@
         <v>0</v>
       </c>
       <c r="U92">
-        <f>IF(H92&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C92,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F92)-COUNTIFS($C$2:$C$102,$C92,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F92)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V92">
-        <f>IF(AND(H92="created",T92=0,COUNTIFS($C$2:$C$102,$C92,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F92)&gt;0,COUNTIFS($C$2:$C$102,$C92,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F92)-COUNTIFS($C$2:$C$102,$C92,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F92)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22074,11 +22075,11 @@
         <v>0</v>
       </c>
       <c r="U93">
-        <f>IF(H93&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C93,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F93)-COUNTIFS($C$2:$C$102,$C93,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F93)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V93">
-        <f>IF(AND(H93="created",T93=0,COUNTIFS($C$2:$C$102,$C93,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F93)&gt;0,COUNTIFS($C$2:$C$102,$C93,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F93)-COUNTIFS($C$2:$C$102,$C93,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F93)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22147,11 +22148,11 @@
         <v>0</v>
       </c>
       <c r="U94">
-        <f>IF(H94&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C94,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F94)-COUNTIFS($C$2:$C$102,$C94,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F94)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V94">
-        <f>IF(AND(H94="created",T94=0,COUNTIFS($C$2:$C$102,$C94,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F94)&gt;0,COUNTIFS($C$2:$C$102,$C94,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F94)-COUNTIFS($C$2:$C$102,$C94,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F94)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22220,11 +22221,11 @@
         <v>0</v>
       </c>
       <c r="U95">
-        <f>IF(H95&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C95,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F95)-COUNTIFS($C$2:$C$102,$C95,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F95)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V95">
-        <f>IF(AND(H95="created",T95=0,COUNTIFS($C$2:$C$102,$C95,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F95)&gt;0,COUNTIFS($C$2:$C$102,$C95,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F95)-COUNTIFS($C$2:$C$102,$C95,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F95)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22293,11 +22294,11 @@
         <v>0</v>
       </c>
       <c r="U96">
-        <f>IF(H96&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C96,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F96)-COUNTIFS($C$2:$C$102,$C96,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F96)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V96">
-        <f>IF(AND(H96="created",T96=0,COUNTIFS($C$2:$C$102,$C96,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F96)&gt;0,COUNTIFS($C$2:$C$102,$C96,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F96)-COUNTIFS($C$2:$C$102,$C96,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F96)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22354,11 +22355,11 @@
         <v>1</v>
       </c>
       <c r="U97">
-        <f>IF(H97&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C97,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F97)-COUNTIFS($C$2:$C$102,$C97,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F97)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V97">
-        <f>IF(AND(H97="created",T97=0,COUNTIFS($C$2:$C$102,$C97,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F97)&gt;0,COUNTIFS($C$2:$C$102,$C97,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F97)-COUNTIFS($C$2:$C$102,$C97,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F97)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22427,11 +22428,11 @@
         <v>0</v>
       </c>
       <c r="U98">
-        <f>IF(H98&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C98,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F98)-COUNTIFS($C$2:$C$102,$C98,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F98)=0,1,0))</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="V98">
-        <f>IF(AND(H98="created",T98=0,COUNTIFS($C$2:$C$102,$C98,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F98)&gt;0,COUNTIFS($C$2:$C$102,$C98,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F98)-COUNTIFS($C$2:$C$102,$C98,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F98)=0),1,0)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -22488,11 +22489,11 @@
         <v>1</v>
       </c>
       <c r="U99">
-        <f t="shared" ref="U99:U102" si="0">IF(H99&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F99)-COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F99)=0,1,0))</f>
+        <f t="shared" ref="U99:U102" si="6">IF(H99&lt;&gt;"cancelled",0,IF(COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"created",$F$2:$F$102,"&lt;="&amp;F99)-COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;="&amp;F99)=0,1,0))</f>
         <v>0</v>
       </c>
       <c r="V99">
-        <f t="shared" ref="V99:V102" si="1">IF(AND(H99="created",T99=0,COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F99)&gt;0,COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F99)-COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F99)=0),1,0)</f>
+        <f t="shared" ref="V99:V102" si="7">IF(AND(H99="created",T99=0,COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F99)&gt;0,COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"created",$F$2:$F$102,"&lt;"&amp;F99)-COUNTIFS($C$2:$C$102,$C99,$H$2:$H$102,"cancelled",$F$2:$F$102,"&lt;"&amp;F99)=0),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -22549,11 +22550,11 @@
         <v>1</v>
       </c>
       <c r="U100">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="V100">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -22610,11 +22611,11 @@
         <v>1</v>
       </c>
       <c r="U101">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="V101">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -22683,11 +22684,11 @@
         <v>0</v>
       </c>
       <c r="U102">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="V102">
-        <f t="shared" si="1"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>